<commit_message>
Add cards-feature, columns-media, hero-banner blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 74
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-rich.report.xlsx
+++ b/tools/importer/reports/import-article-rich.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="347">
   <si>
     <t>_reportFile</t>
   </si>
@@ -79,7 +79,7 @@
     <t>info-page</t>
   </si>
   <si>
-    <t>2026-10-06T21:02:53.568Z</t>
+    <t>2026-10-07T15:02:11.620Z</t>
   </si>
   <si>
     <t>About us – Bradesco Bank</t>
@@ -97,7 +97,7 @@
     <t>listing</t>
   </si>
   <si>
-    <t>2026-10-06T21:08:26.689Z</t>
+    <t>2026-10-07T15:06:24.121Z</t>
   </si>
   <si>
     <t>Articles Archive – Bradesco Bank</t>
@@ -115,7 +115,7 @@
     <t>en/bank-holidays</t>
   </si>
   <si>
-    <t>2026-10-06T21:04:11.114Z</t>
+    <t>2026-10-07T15:03:28.609Z</t>
   </si>
   <si>
     <t>Bank Holidays – Bradesco Bank</t>
@@ -130,7 +130,7 @@
     <t>en/bradesco-lounge</t>
   </si>
   <si>
-    <t>2026-10-06T21:04:23.137Z</t>
+    <t>2026-10-07T15:03:37.726Z</t>
   </si>
   <si>
     <t>Bradesco Lounge – Bradesco Bank</t>
@@ -151,7 +151,7 @@
     <t>landing</t>
   </si>
   <si>
-    <t>2026-10-06T21:01:37.689Z</t>
+    <t>2026-10-07T14:59:52.918Z</t>
   </si>
   <si>
     <t>Careers – Bradesco Bank</t>
@@ -169,7 +169,7 @@
     <t>en/certificate-of-deposit-bradesco</t>
   </si>
   <si>
-    <t>2026-10-06T21:00:46.965Z</t>
+    <t>2026-10-07T14:58:58.176Z</t>
   </si>
   <si>
     <t>CDB – Bradesco Bank</t>
@@ -187,7 +187,7 @@
     <t>en/corporate</t>
   </si>
   <si>
-    <t>2026-10-06T20:59:05.643Z</t>
+    <t>2026-10-07T14:57:21.711Z</t>
   </si>
   <si>
     <t>Business Corporate – Bradesco Bank</t>
@@ -202,7 +202,7 @@
     <t>en/cra-public-file</t>
   </si>
   <si>
-    <t>2026-10-06T21:05:05.773Z</t>
+    <t>2026-10-07T15:04:21.625Z</t>
   </si>
   <si>
     <t>CRA Public File – Bradesco Bank</t>
@@ -220,7 +220,7 @@
     <t>en/credit-card-signature-gold</t>
   </si>
   <si>
-    <t>2026-10-06T21:00:35.845Z</t>
+    <t>2026-10-07T14:58:49.935Z</t>
   </si>
   <si>
     <t>Signature &amp; Gold – Bradesco Bank</t>
@@ -238,7 +238,7 @@
     <t>en/credit-cards</t>
   </si>
   <si>
-    <t>2026-10-06T21:00:19.436Z</t>
+    <t>2026-10-07T14:58:32.935Z</t>
   </si>
   <si>
     <t>Credit Cards – Bradesco Bank</t>
@@ -259,7 +259,7 @@
     <t>article-rich</t>
   </si>
   <si>
-    <t>2026-10-06T21:20:26.778Z</t>
+    <t>2026-10-07T15:09:09.430Z</t>
   </si>
   <si>
     <t>Exploring Investment Products in the U.S. – Bradesco Bank</t>
@@ -313,7 +313,7 @@
     <t>en/help</t>
   </si>
   <si>
-    <t>2026-10-06T21:04:00.977Z</t>
+    <t>2026-10-07T15:03:18.757Z</t>
   </si>
   <si>
     <t>How Can We Help? – Bradesco Bank</t>
@@ -361,7 +361,7 @@
     <t>en/insights-archive</t>
   </si>
   <si>
-    <t>2026-10-06T21:08:46.097Z</t>
+    <t>2026-10-07T15:06:46.819Z</t>
   </si>
   <si>
     <t>Insights Archive – Bradesco Bank</t>
@@ -379,7 +379,7 @@
     <t>en/institutional</t>
   </si>
   <si>
-    <t>2026-10-06T21:03:50.041Z</t>
+    <t>2026-10-07T15:03:08.851Z</t>
   </si>
   <si>
     <t>Business – Institutional – Bradesco Bank</t>
@@ -397,7 +397,7 @@
     <t>en/investing-for-different-client-profiles</t>
   </si>
   <si>
-    <t>2026-10-06T21:20:41.691Z</t>
+    <t>2026-10-07T15:09:25.575Z</t>
   </si>
   <si>
     <t>Investing for Different Client Profiles – Bradesco Bank</t>
@@ -430,7 +430,7 @@
     <t>en/investments-content</t>
   </si>
   <si>
-    <t>2026-10-06T21:08:04.440Z</t>
+    <t>2026-10-07T15:05:57.982Z</t>
   </si>
   <si>
     <t>Investments Content – Bradesco Bank</t>
@@ -475,7 +475,7 @@
     <t>en/other-disclosures</t>
   </si>
   <si>
-    <t>2026-10-06T21:04:55.089Z</t>
+    <t>2026-10-07T15:04:10.484Z</t>
   </si>
   <si>
     <t>Other disclosures – Bradesco Bank</t>
@@ -493,7 +493,7 @@
     <t>en/personal-bank</t>
   </si>
   <si>
-    <t>2026-10-06T20:57:54.040Z</t>
+    <t>2026-10-07T14:55:26.660Z</t>
   </si>
   <si>
     <t>Personal Bank – Bradesco Bank</t>
@@ -526,7 +526,7 @@
     <t>en/privacy-and-cookies</t>
   </si>
   <si>
-    <t>2026-10-06T21:04:43.643Z</t>
+    <t>2026-10-07T15:03:57.994Z</t>
   </si>
   <si>
     <t>Privacy and Cookies – Bradesco Bank</t>
@@ -544,7 +544,7 @@
     <t>en/private-bank</t>
   </si>
   <si>
-    <t>2026-10-06T20:58:51.989Z</t>
+    <t>2026-10-07T14:56:24.261Z</t>
   </si>
   <si>
     <t>Private Bank – Bradesco Bank</t>
@@ -562,7 +562,7 @@
     <t>en/real-estate</t>
   </si>
   <si>
-    <t>2026-10-06T21:00:05.435Z</t>
+    <t>2026-10-07T14:58:21.352Z</t>
   </si>
   <si>
     <t>Real Estate – Bradesco Bank</t>
@@ -598,7 +598,7 @@
     <t>en/security</t>
   </si>
   <si>
-    <t>2026-10-06T21:04:33.004Z</t>
+    <t>2026-10-07T15:03:46.522Z</t>
   </si>
   <si>
     <t>Security – Bradesco Bank</t>
@@ -616,7 +616,7 @@
     <t>en/the-power-of-compounding</t>
   </si>
   <si>
-    <t>2026-10-06T21:20:51.373Z</t>
+    <t>2026-10-07T15:09:35.826Z</t>
   </si>
   <si>
     <t>The Power of Compounding – Bradesco Bank</t>
@@ -655,6 +655,57 @@
     <t>https://bradescobank.com/en/u-s-stocks/</t>
   </si>
   <si>
+    <t>en/visa-gold-activation.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","cards-feature","columns-media"]</t>
+  </si>
+  <si>
+    <t>en/visa-gold-activation</t>
+  </si>
+  <si>
+    <t>card-activation</t>
+  </si>
+  <si>
+    <t>2026-10-07T14:47:34.330Z</t>
+  </si>
+  <si>
+    <t>Gold Activation – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/visa-gold-activation/</t>
+  </si>
+  <si>
+    <t>en/visa-infinite-activation.report.json</t>
+  </si>
+  <si>
+    <t>en/visa-infinite-activation</t>
+  </si>
+  <si>
+    <t>2026-10-07T14:47:44.501Z</t>
+  </si>
+  <si>
+    <t>Infinite Activation – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/visa-infinite-activation/</t>
+  </si>
+  <si>
+    <t>en/visa-signature-activation.report.json</t>
+  </si>
+  <si>
+    <t>en/visa-signature-activation</t>
+  </si>
+  <si>
+    <t>2026-10-07T14:47:54.545Z</t>
+  </si>
+  <si>
+    <t>Signature Activation – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/visa-signature-activation/</t>
+  </si>
+  <si>
     <t>en/what-are-asset-allocation-and-diversification.report.json</t>
   </si>
   <si>
@@ -694,7 +745,7 @@
     <t>en/zelle</t>
   </si>
   <si>
-    <t>2026-10-06T21:00:57.523Z</t>
+    <t>2026-10-07T14:59:10.709Z</t>
   </si>
   <si>
     <t>Zelle – Bradesco Bank</t>
@@ -703,6 +754,54 @@
     <t>https://bradescobank.com/en/zelle/</t>
   </si>
   <si>
+    <t>en/category/educational.report.json</t>
+  </si>
+  <si>
+    <t>en/category/educational</t>
+  </si>
+  <si>
+    <t>category-listing</t>
+  </si>
+  <si>
+    <t>2026-10-07T15:07:23.005Z</t>
+  </si>
+  <si>
+    <t>Educational – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/category/educational/</t>
+  </si>
+  <si>
+    <t>en/category/market-insight.report.json</t>
+  </si>
+  <si>
+    <t>en/category/market-insight</t>
+  </si>
+  <si>
+    <t>2026-10-07T15:07:46.588Z</t>
+  </si>
+  <si>
+    <t>Market Insight – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/category/market-insight/</t>
+  </si>
+  <si>
+    <t>en/category/videos.report.json</t>
+  </si>
+  <si>
+    <t>en/category/videos</t>
+  </si>
+  <si>
+    <t>2026-10-07T15:08:08.988Z</t>
+  </si>
+  <si>
+    <t>Videos – Bradesco Bank</t>
+  </si>
+  <si>
+    <t>https://bradescobank.com/en/category/videos/</t>
+  </si>
+  <si>
     <t>en/credit-card/visa-infinite.report.json</t>
   </si>
   <si>
@@ -712,7 +811,7 @@
     <t>en/credit-card/visa-infinite</t>
   </si>
   <si>
-    <t>2026-10-06T21:01:08.193Z</t>
+    <t>2026-10-07T14:59:21.291Z</t>
   </si>
   <si>
     <t>Visa Infinite – Bradesco Bank</t>
@@ -730,7 +829,7 @@
     <t>en/investments-content/bradesco-investments-app</t>
   </si>
   <si>
-    <t>2026-10-06T21:01:28.750Z</t>
+    <t>2026-10-07T14:59:42.928Z</t>
   </si>
   <si>
     <t>Bradesco Investments App – Bradesco Bank</t>
@@ -748,7 +847,7 @@
     <t>en/investments-content/saved-articles</t>
   </si>
   <si>
-    <t>2026-10-06T21:08:55.045Z</t>
+    <t>2026-10-07T15:06:58.400Z</t>
   </si>
   <si>
     <t>Saved Articles – Bradesco Bank</t>
@@ -769,7 +868,7 @@
     <t>faq-hub</t>
   </si>
   <si>
-    <t>2026-10-06T21:06:56.817Z</t>
+    <t>2026-10-07T15:08:32.879Z</t>
   </si>
   <si>
     <t>FAQ – Bradesco Bank</t>
@@ -787,7 +886,7 @@
     <t>en/personal-bank/investments</t>
   </si>
   <si>
-    <t>2026-10-06T21:01:17.563Z</t>
+    <t>2026-10-07T14:59:31.779Z</t>
   </si>
   <si>
     <t>Investments – Bradesco Bank</t>
@@ -808,7 +907,7 @@
     <t>en/careers/fragments/internship</t>
   </si>
   <si>
-    <t>2026-10-06T21:02:42.494Z</t>
+    <t>2026-10-07T15:01:08.889Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/careers/?fragment=internship</t>
@@ -826,7 +925,7 @@
     <t>en/careers/fragments/jobs</t>
   </si>
   <si>
-    <t>2026-10-06T21:02:32.519Z</t>
+    <t>2026-10-07T15:00:59.292Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/careers/?fragment=jobs</t>
@@ -838,7 +937,7 @@
     <t>en/personal-bank/investments/faq</t>
   </si>
   <si>
-    <t>2026-10-06T21:07:21.777Z</t>
+    <t>2026-10-07T15:08:57.756Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/personal-bank/investments/faq/</t>
@@ -856,7 +955,7 @@
     <t>en/privacy-and-cookies/fragments/bradesco-investments-privacy-notice</t>
   </si>
   <si>
-    <t>2026-10-06T21:05:34.672Z</t>
+    <t>2026-10-07T15:04:50.169Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=bradesco-investments-privacy-notice</t>
@@ -874,7 +973,7 @@
     <t>en/privacy-and-cookies/fragments/california-consumer-privacy-act-ccpa</t>
   </si>
   <si>
-    <t>2026-10-06T21:05:56.897Z</t>
+    <t>2026-10-07T15:05:13.747Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=california-consumer-privacy-act-ccpa</t>
@@ -889,7 +988,7 @@
     <t>en/privacy-and-cookies/fragments/childrens-privacy-policy</t>
   </si>
   <si>
-    <t>2026-10-06T21:06:09.321Z</t>
+    <t>2026-10-07T15:05:23.838Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=childrens-privacy-policy</t>
@@ -904,7 +1003,7 @@
     <t>en/privacy-and-cookies/fragments/consumer-privacy-notice</t>
   </si>
   <si>
-    <t>2026-10-06T21:05:23.389Z</t>
+    <t>2026-10-07T15:04:38.920Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=consumer-privacy-notice</t>
@@ -919,7 +1018,7 @@
     <t>en/privacy-and-cookies/fragments/online-privacy-notice</t>
   </si>
   <si>
-    <t>2026-10-06T21:05:46.337Z</t>
+    <t>2026-10-07T15:05:01.049Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=online-privacy-notice</t>
@@ -934,7 +1033,7 @@
     <t>en/privacy-and-cookies/fragments/others</t>
   </si>
   <si>
-    <t>2026-10-06T21:06:31.843Z</t>
+    <t>2026-10-07T15:05:45.254Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=others</t>
@@ -949,7 +1048,7 @@
     <t>en/privacy-and-cookies/fragments/sms-terms-of-service</t>
   </si>
   <si>
-    <t>2026-10-06T21:06:21.557Z</t>
+    <t>2026-10-07T15:05:33.495Z</t>
   </si>
   <si>
     <t>https://bradescobank.com/en/privacy-and-cookies/?fragment=sms-terms-of-service</t>
@@ -1341,13 +1440,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
     <col min="4" max="4" width="50" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="9" width="50" customWidth="1"/>
   </cols>
@@ -2401,94 +2500,94 @@
         <v>214</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
+        <v>215</v>
       </c>
       <c r="C37" t="s">
         <v>11</v>
       </c>
       <c r="D37" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E37" t="s">
         <v>13</v>
       </c>
       <c r="F37" t="s">
-        <v>88</v>
+        <v>217</v>
       </c>
       <c r="G37" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="H37" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I37" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
+        <v>215</v>
       </c>
       <c r="C38" t="s">
         <v>11</v>
       </c>
       <c r="D38" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E38" t="s">
         <v>13</v>
       </c>
       <c r="F38" t="s">
-        <v>88</v>
+        <v>217</v>
       </c>
       <c r="G38" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="H38" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I38" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B39" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C39" t="s">
         <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E39" t="s">
         <v>13</v>
       </c>
       <c r="F39" t="s">
-        <v>45</v>
+        <v>217</v>
       </c>
       <c r="G39" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H39" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I39" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B40" t="s">
-        <v>231</v>
+        <v>86</v>
       </c>
       <c r="C40" t="s">
         <v>11</v>
@@ -2500,7 +2599,7 @@
         <v>13</v>
       </c>
       <c r="F40" t="s">
-        <v>45</v>
+        <v>88</v>
       </c>
       <c r="G40" t="s">
         <v>233</v>
@@ -2517,158 +2616,158 @@
         <v>236</v>
       </c>
       <c r="B41" t="s">
+        <v>86</v>
+      </c>
+      <c r="C41" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" t="s">
         <v>237</v>
       </c>
-      <c r="C41" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" t="s">
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41" t="s">
+        <v>88</v>
+      </c>
+      <c r="G41" t="s">
         <v>238</v>
       </c>
-      <c r="E41" t="s">
-        <v>13</v>
-      </c>
-      <c r="F41" t="s">
-        <v>45</v>
-      </c>
-      <c r="G41" t="s">
+      <c r="H41" t="s">
         <v>239</v>
       </c>
-      <c r="H41" t="s">
+      <c r="I41" t="s">
         <v>240</v>
-      </c>
-      <c r="I41" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>241</v>
+      </c>
+      <c r="B42" t="s">
         <v>242</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" t="s">
         <v>243</v>
       </c>
-      <c r="C42" t="s">
-        <v>11</v>
-      </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
+        <v>13</v>
+      </c>
+      <c r="F42" t="s">
+        <v>45</v>
+      </c>
+      <c r="G42" t="s">
         <v>244</v>
       </c>
-      <c r="E42" t="s">
-        <v>13</v>
-      </c>
-      <c r="F42" t="s">
-        <v>27</v>
-      </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>245</v>
       </c>
-      <c r="H42" t="s">
+      <c r="I42" t="s">
         <v>246</v>
-      </c>
-      <c r="I42" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>247</v>
+      </c>
+      <c r="B43" t="s">
+        <v>19</v>
+      </c>
+      <c r="C43" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" t="s">
         <v>248</v>
       </c>
-      <c r="B43" t="s">
+      <c r="E43" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" t="s">
         <v>249</v>
       </c>
-      <c r="C43" t="s">
-        <v>11</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="G43" t="s">
         <v>250</v>
       </c>
-      <c r="E43" t="s">
-        <v>13</v>
-      </c>
-      <c r="F43" t="s">
+      <c r="H43" t="s">
         <v>251</v>
       </c>
-      <c r="G43" t="s">
+      <c r="I43" t="s">
         <v>252</v>
-      </c>
-      <c r="H43" t="s">
-        <v>253</v>
-      </c>
-      <c r="I43" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>253</v>
+      </c>
+      <c r="B44" t="s">
+        <v>19</v>
+      </c>
+      <c r="C44" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" t="s">
+        <v>254</v>
+      </c>
+      <c r="E44" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" t="s">
+        <v>249</v>
+      </c>
+      <c r="G44" t="s">
         <v>255</v>
       </c>
-      <c r="B44" t="s">
+      <c r="H44" t="s">
         <v>256</v>
       </c>
-      <c r="C44" t="s">
-        <v>11</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="I44" t="s">
         <v>257</v>
-      </c>
-      <c r="E44" t="s">
-        <v>13</v>
-      </c>
-      <c r="F44" t="s">
-        <v>45</v>
-      </c>
-      <c r="G44" t="s">
-        <v>258</v>
-      </c>
-      <c r="H44" t="s">
-        <v>259</v>
-      </c>
-      <c r="I44" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>258</v>
+      </c>
+      <c r="B45" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" t="s">
+        <v>259</v>
+      </c>
+      <c r="E45" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" t="s">
+        <v>249</v>
+      </c>
+      <c r="G45" t="s">
+        <v>260</v>
+      </c>
+      <c r="H45" t="s">
         <v>261</v>
       </c>
-      <c r="B45" t="s">
+      <c r="I45" t="s">
         <v>262</v>
-      </c>
-      <c r="C45" t="s">
-        <v>263</v>
-      </c>
-      <c r="D45" t="s">
-        <v>264</v>
-      </c>
-      <c r="E45" t="s">
-        <v>13</v>
-      </c>
-      <c r="F45" t="s">
-        <v>45</v>
-      </c>
-      <c r="G45" t="s">
-        <v>265</v>
-      </c>
-      <c r="H45" t="s">
-        <v>47</v>
-      </c>
-      <c r="I45" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B46" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C46" t="s">
-        <v>269</v>
+        <v>11</v>
       </c>
       <c r="D46" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="E46" t="s">
         <v>13</v>
@@ -2677,126 +2776,126 @@
         <v>45</v>
       </c>
       <c r="G46" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="H46" t="s">
-        <v>47</v>
+        <v>267</v>
       </c>
       <c r="I46" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>269</v>
+      </c>
+      <c r="B47" t="s">
+        <v>270</v>
+      </c>
+      <c r="C47" t="s">
+        <v>11</v>
+      </c>
+      <c r="D47" t="s">
+        <v>271</v>
+      </c>
+      <c r="E47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" t="s">
+        <v>45</v>
+      </c>
+      <c r="G47" t="s">
+        <v>272</v>
+      </c>
+      <c r="H47" t="s">
         <v>273</v>
       </c>
-      <c r="B47" t="s">
-        <v>249</v>
-      </c>
-      <c r="C47" t="s">
-        <v>11</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="I47" t="s">
         <v>274</v>
-      </c>
-      <c r="E47" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" t="s">
-        <v>251</v>
-      </c>
-      <c r="G47" t="s">
-        <v>275</v>
-      </c>
-      <c r="H47" t="s">
-        <v>253</v>
-      </c>
-      <c r="I47" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>275</v>
+      </c>
+      <c r="B48" t="s">
+        <v>276</v>
+      </c>
+      <c r="C48" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" t="s">
         <v>277</v>
       </c>
-      <c r="B48" t="s">
+      <c r="E48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" t="s">
+        <v>27</v>
+      </c>
+      <c r="G48" t="s">
         <v>278</v>
       </c>
-      <c r="C48" t="s">
+      <c r="H48" t="s">
         <v>279</v>
       </c>
-      <c r="D48" t="s">
+      <c r="I48" t="s">
         <v>280</v>
-      </c>
-      <c r="E48" t="s">
-        <v>13</v>
-      </c>
-      <c r="F48" t="s">
-        <v>21</v>
-      </c>
-      <c r="G48" t="s">
-        <v>281</v>
-      </c>
-      <c r="H48" t="s">
-        <v>172</v>
-      </c>
-      <c r="I48" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>281</v>
+      </c>
+      <c r="B49" t="s">
+        <v>282</v>
+      </c>
+      <c r="C49" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" t="s">
         <v>283</v>
       </c>
-      <c r="B49" t="s">
+      <c r="E49" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" t="s">
         <v>284</v>
       </c>
-      <c r="C49" t="s">
+      <c r="G49" t="s">
         <v>285</v>
       </c>
-      <c r="D49" t="s">
+      <c r="H49" t="s">
         <v>286</v>
       </c>
-      <c r="E49" t="s">
-        <v>13</v>
-      </c>
-      <c r="F49" t="s">
-        <v>21</v>
-      </c>
-      <c r="G49" t="s">
+      <c r="I49" t="s">
         <v>287</v>
-      </c>
-      <c r="H49" t="s">
-        <v>172</v>
-      </c>
-      <c r="I49" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>288</v>
+      </c>
+      <c r="B50" t="s">
         <v>289</v>
       </c>
-      <c r="B50" t="s">
-        <v>268</v>
-      </c>
       <c r="C50" t="s">
+        <v>11</v>
+      </c>
+      <c r="D50" t="s">
         <v>290</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" t="s">
+        <v>45</v>
+      </c>
+      <c r="G50" t="s">
         <v>291</v>
       </c>
-      <c r="E50" t="s">
-        <v>13</v>
-      </c>
-      <c r="F50" t="s">
-        <v>21</v>
-      </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>292</v>
-      </c>
-      <c r="H50" t="s">
-        <v>172</v>
       </c>
       <c r="I50" t="s">
         <v>293</v>
@@ -2807,100 +2906,100 @@
         <v>294</v>
       </c>
       <c r="B51" t="s">
-        <v>278</v>
+        <v>295</v>
       </c>
       <c r="C51" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D51" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E51" t="s">
         <v>13</v>
       </c>
       <c r="F51" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="G51" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="H51" t="s">
-        <v>172</v>
+        <v>47</v>
       </c>
       <c r="I51" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B52" t="s">
-        <v>268</v>
+        <v>301</v>
       </c>
       <c r="C52" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D52" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E52" t="s">
         <v>13</v>
       </c>
       <c r="F52" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="G52" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H52" t="s">
-        <v>172</v>
+        <v>47</v>
       </c>
       <c r="I52" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B53" t="s">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="C53" t="s">
-        <v>305</v>
+        <v>11</v>
       </c>
       <c r="D53" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E53" t="s">
         <v>13</v>
       </c>
       <c r="F53" t="s">
-        <v>21</v>
+        <v>284</v>
       </c>
       <c r="G53" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H53" t="s">
-        <v>172</v>
+        <v>286</v>
       </c>
       <c r="I53" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B54" t="s">
-        <v>268</v>
+        <v>311</v>
       </c>
       <c r="C54" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D54" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E54" t="s">
         <v>13</v>
@@ -2909,13 +3008,187 @@
         <v>21</v>
       </c>
       <c r="G54" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="H54" t="s">
         <v>172</v>
       </c>
       <c r="I54" t="s">
-        <v>313</v>
+        <v>315</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>316</v>
+      </c>
+      <c r="B55" t="s">
+        <v>317</v>
+      </c>
+      <c r="C55" t="s">
+        <v>318</v>
+      </c>
+      <c r="D55" t="s">
+        <v>319</v>
+      </c>
+      <c r="E55" t="s">
+        <v>13</v>
+      </c>
+      <c r="F55" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" t="s">
+        <v>320</v>
+      </c>
+      <c r="H55" t="s">
+        <v>172</v>
+      </c>
+      <c r="I55" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>322</v>
+      </c>
+      <c r="B56" t="s">
+        <v>301</v>
+      </c>
+      <c r="C56" t="s">
+        <v>323</v>
+      </c>
+      <c r="D56" t="s">
+        <v>324</v>
+      </c>
+      <c r="E56" t="s">
+        <v>13</v>
+      </c>
+      <c r="F56" t="s">
+        <v>21</v>
+      </c>
+      <c r="G56" t="s">
+        <v>325</v>
+      </c>
+      <c r="H56" t="s">
+        <v>172</v>
+      </c>
+      <c r="I56" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>327</v>
+      </c>
+      <c r="B57" t="s">
+        <v>311</v>
+      </c>
+      <c r="C57" t="s">
+        <v>328</v>
+      </c>
+      <c r="D57" t="s">
+        <v>329</v>
+      </c>
+      <c r="E57" t="s">
+        <v>13</v>
+      </c>
+      <c r="F57" t="s">
+        <v>21</v>
+      </c>
+      <c r="G57" t="s">
+        <v>330</v>
+      </c>
+      <c r="H57" t="s">
+        <v>172</v>
+      </c>
+      <c r="I57" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>332</v>
+      </c>
+      <c r="B58" t="s">
+        <v>301</v>
+      </c>
+      <c r="C58" t="s">
+        <v>333</v>
+      </c>
+      <c r="D58" t="s">
+        <v>334</v>
+      </c>
+      <c r="E58" t="s">
+        <v>13</v>
+      </c>
+      <c r="F58" t="s">
+        <v>21</v>
+      </c>
+      <c r="G58" t="s">
+        <v>335</v>
+      </c>
+      <c r="H58" t="s">
+        <v>172</v>
+      </c>
+      <c r="I58" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>337</v>
+      </c>
+      <c r="B59" t="s">
+        <v>301</v>
+      </c>
+      <c r="C59" t="s">
+        <v>338</v>
+      </c>
+      <c r="D59" t="s">
+        <v>339</v>
+      </c>
+      <c r="E59" t="s">
+        <v>13</v>
+      </c>
+      <c r="F59" t="s">
+        <v>21</v>
+      </c>
+      <c r="G59" t="s">
+        <v>340</v>
+      </c>
+      <c r="H59" t="s">
+        <v>172</v>
+      </c>
+      <c r="I59" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>342</v>
+      </c>
+      <c r="B60" t="s">
+        <v>301</v>
+      </c>
+      <c r="C60" t="s">
+        <v>343</v>
+      </c>
+      <c r="D60" t="s">
+        <v>344</v>
+      </c>
+      <c r="E60" t="s">
+        <v>13</v>
+      </c>
+      <c r="F60" t="s">
+        <v>21</v>
+      </c>
+      <c r="G60" t="s">
+        <v>345</v>
+      </c>
+      <c r="H60" t="s">
+        <v>172</v>
+      </c>
+      <c r="I60" t="s">
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>